<commit_message>
Add simulation performance and financial metrics
</commit_message>
<xml_diff>
--- a/static/Plantilla_simulacion_excedentes.xlsx
+++ b/static/Plantilla_simulacion_excedentes.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="Rb429f53838d747f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuración" sheetId="2" r:id="Rb564659683c147e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumo horario" sheetId="3" r:id="Ra7dd0eeb4a074cb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generación PVSyst" sheetId="4" r:id="Re13317b5a5b7430c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfil PVSyst" sheetId="5" r:id="R1717ac302a714368"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R17ccf67432d24982"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuración" sheetId="2" r:id="R02ed9f42c0614f8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumo horario" sheetId="3" r:id="R4edba76ee9454c3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generación PVSyst" sheetId="4" r:id="R7a769f0060494f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfil PVSyst" sheetId="5" r:id="R13882c0a788f40aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,12 +17,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.0"/>
     <x:numFmt numFmtId="202" formatCode="dd/mm/yyyy"/>
     <x:numFmt numFmtId="203" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="204" formatCode="0.0%"/>
+    <x:numFmt numFmtId="205" formatCode="#,##0"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -64,7 +65,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -89,6 +90,36 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF3CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF16835C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF16835C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF153D35"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF153D35"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -240,7 +271,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="66">
+  <x:cellXfs count="92">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -353,6 +384,56 @@
     <x:xf numFmtId="201" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -11859,13 +11940,13 @@
       <x:c r="Z1" s="1"/>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
-      <x:c r="A2" s="4" t="str">
+      <x:c r="A2" s="80" t="str">
         <x:v>Configuración de la planta</x:v>
       </x:c>
-      <x:c r="B2" s="4" t="str">
+      <x:c r="B2" s="80" t="str">
         <x:v>Configuración de la planta</x:v>
       </x:c>
-      <x:c r="C2" s="4" t="str">
+      <x:c r="C2" s="80" t="str">
         <x:v>Configuración de la planta</x:v>
       </x:c>
       <x:c r="D2" s="4" t="str">
@@ -11923,13 +12004,13 @@
       <x:c r="Z3" s="1"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="60" t="str">
+      <x:c r="A4" s="85" t="str">
         <x:v>Campo</x:v>
       </x:c>
-      <x:c r="B4" s="60" t="str">
+      <x:c r="B4" s="85" t="str">
         <x:v>Valor</x:v>
       </x:c>
-      <x:c r="C4" s="60" t="str">
+      <x:c r="C4" s="85" t="str">
         <x:v>Uso en la aplicación</x:v>
       </x:c>
       <x:c r="D4" s="1"/>
@@ -11960,7 +12041,7 @@
       <x:c r="A5" s="63" t="str">
         <x:v>Nombre de la planta</x:v>
       </x:c>
-      <x:c r="B5" s="64" t="str"/>
+      <x:c r="B5" s="86" t="str"/>
       <x:c r="C5" s="63" t="str">
         <x:v>Identifica esta fuente en el selector.</x:v>
       </x:c>
@@ -11992,7 +12073,7 @@
       <x:c r="A6" s="63" t="str">
         <x:v>Año de consumo</x:v>
       </x:c>
-      <x:c r="B6" s="64" t="str"/>
+      <x:c r="B6" s="86" t="str"/>
       <x:c r="C6" s="63" t="str">
         <x:v>Debe coincidir con las fechas de Consumo horario.</x:v>
       </x:c>
@@ -12024,9 +12105,9 @@
       <x:c r="A7" s="63" t="str">
         <x:v>Capacidad FV instalada (kWp)</x:v>
       </x:c>
-      <x:c r="B7" s="65" t="str"/>
+      <x:c r="B7" s="87" t="str"/>
       <x:c r="C7" s="63" t="str">
-        <x:v>Dato de referencia para revisión técnica. No modifica el cálculo actual.</x:v>
+        <x:v>Referencia para el desempeño técnico.</x:v>
       </x:c>
       <x:c r="D7" s="1"/>
       <x:c r="E7" s="1"/>
@@ -12053,9 +12134,13 @@
       <x:c r="Z7" s="1"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8"/>
-      <x:c r="B8"/>
-      <x:c r="C8"/>
+      <x:c r="A8" s="63" t="str">
+        <x:v>Tarifa de energía evitada (COP/kWh)</x:v>
+      </x:c>
+      <x:c r="B8" s="88" t="str"/>
+      <x:c r="C8" s="63" t="str">
+        <x:v>Convierte la desviación energética estimada a COP.</x:v>
+      </x:c>
       <x:c r="D8" s="1"/>
       <x:c r="E8" s="1"/>
       <x:c r="F8" s="1"/>
@@ -23058,7 +23143,7 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A2:D2"/>
+    <x:mergeCell ref="A2:C2"/>
   </x:mergeCells>
   <x:dataValidations count="1">
     <x:dataValidation type="decimal" operator="between" sqref="B7">
@@ -34426,22 +34511,23 @@
     <x:col min="2" max="2" width="19" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="19" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="80" t="str">
         <x:v>Producción mensual estimada PVSyst</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="80" t="str">
         <x:v>Producción mensual estimada PVSyst</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="80" t="str">
         <x:v>Producción mensual estimada PVSyst</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="80" t="str">
         <x:v>Producción mensual estimada PVSyst</x:v>
       </x:c>
-      <x:c r="E1" s="1"/>
+      <x:c r="E1" s="80"/>
       <x:c r="F1" s="1"/>
       <x:c r="G1" s="1"/>
       <x:c r="H1" s="1"/>
@@ -34535,7 +34621,9 @@
       <x:c r="D4" s="12" t="str">
         <x:v>PR (%)</x:v>
       </x:c>
-      <x:c r="E4" s="1"/>
+      <x:c r="E4" s="85" t="str">
+        <x:v>Generación real (kWh)</x:v>
+      </x:c>
       <x:c r="F4" s="1"/>
       <x:c r="G4" s="1"/>
       <x:c r="H4" s="1"/>
@@ -34565,7 +34653,7 @@
       <x:c r="B5" s="54"/>
       <x:c r="C5" s="54"/>
       <x:c r="D5" s="55"/>
-      <x:c r="E5" s="1"/>
+      <x:c r="E5" s="91"/>
       <x:c r="F5" s="1"/>
       <x:c r="G5" s="1"/>
       <x:c r="H5" s="1"/>
@@ -34595,7 +34683,7 @@
       <x:c r="B6" s="54"/>
       <x:c r="C6" s="54"/>
       <x:c r="D6" s="55"/>
-      <x:c r="E6" s="1"/>
+      <x:c r="E6" s="91"/>
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
       <x:c r="H6" s="1"/>
@@ -34625,7 +34713,7 @@
       <x:c r="B7" s="54"/>
       <x:c r="C7" s="54"/>
       <x:c r="D7" s="55"/>
-      <x:c r="E7" s="1"/>
+      <x:c r="E7" s="91"/>
       <x:c r="F7" s="1"/>
       <x:c r="G7" s="1"/>
       <x:c r="H7" s="1"/>
@@ -34655,7 +34743,7 @@
       <x:c r="B8" s="54"/>
       <x:c r="C8" s="54"/>
       <x:c r="D8" s="55"/>
-      <x:c r="E8" s="1"/>
+      <x:c r="E8" s="91"/>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
       <x:c r="H8" s="1"/>
@@ -34685,7 +34773,7 @@
       <x:c r="B9" s="54"/>
       <x:c r="C9" s="54"/>
       <x:c r="D9" s="55"/>
-      <x:c r="E9" s="1"/>
+      <x:c r="E9" s="91"/>
       <x:c r="F9" s="1"/>
       <x:c r="G9" s="1"/>
       <x:c r="H9" s="1"/>
@@ -34715,7 +34803,7 @@
       <x:c r="B10" s="54"/>
       <x:c r="C10" s="54"/>
       <x:c r="D10" s="55"/>
-      <x:c r="E10" s="1"/>
+      <x:c r="E10" s="91"/>
       <x:c r="F10" s="1"/>
       <x:c r="G10" s="1"/>
       <x:c r="H10" s="1"/>
@@ -34745,7 +34833,7 @@
       <x:c r="B11" s="54"/>
       <x:c r="C11" s="54"/>
       <x:c r="D11" s="55"/>
-      <x:c r="E11" s="1"/>
+      <x:c r="E11" s="91"/>
       <x:c r="F11" s="1"/>
       <x:c r="G11" s="1"/>
       <x:c r="H11" s="1"/>
@@ -34775,7 +34863,7 @@
       <x:c r="B12" s="54"/>
       <x:c r="C12" s="54"/>
       <x:c r="D12" s="55"/>
-      <x:c r="E12" s="1"/>
+      <x:c r="E12" s="91"/>
       <x:c r="F12" s="1"/>
       <x:c r="G12" s="1"/>
       <x:c r="H12" s="1"/>
@@ -34805,7 +34893,7 @@
       <x:c r="B13" s="54"/>
       <x:c r="C13" s="54"/>
       <x:c r="D13" s="55"/>
-      <x:c r="E13" s="1"/>
+      <x:c r="E13" s="91"/>
       <x:c r="F13" s="1"/>
       <x:c r="G13" s="1"/>
       <x:c r="H13" s="1"/>
@@ -34835,7 +34923,7 @@
       <x:c r="B14" s="54"/>
       <x:c r="C14" s="54"/>
       <x:c r="D14" s="55"/>
-      <x:c r="E14" s="1"/>
+      <x:c r="E14" s="91"/>
       <x:c r="F14" s="1"/>
       <x:c r="G14" s="1"/>
       <x:c r="H14" s="1"/>
@@ -34865,7 +34953,7 @@
       <x:c r="B15" s="54"/>
       <x:c r="C15" s="54"/>
       <x:c r="D15" s="55"/>
-      <x:c r="E15" s="1"/>
+      <x:c r="E15" s="91"/>
       <x:c r="F15" s="1"/>
       <x:c r="G15" s="1"/>
       <x:c r="H15" s="1"/>
@@ -34895,7 +34983,7 @@
       <x:c r="B16" s="54"/>
       <x:c r="C16" s="54"/>
       <x:c r="D16" s="55"/>
-      <x:c r="E16" s="1"/>
+      <x:c r="E16" s="91"/>
       <x:c r="F16" s="1"/>
       <x:c r="G16" s="1"/>
       <x:c r="H16" s="1"/>
@@ -45672,8 +45760,8 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:D1"/>
     <x:mergeCell ref="A2:D2"/>
+    <x:mergeCell ref="A1:E1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Align simulation with zero export scenarios
</commit_message>
<xml_diff>
--- a/static/Plantilla_simulacion_excedentes.xlsx
+++ b/static/Plantilla_simulacion_excedentes.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R17ccf67432d24982"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuración" sheetId="2" r:id="R02ed9f42c0614f8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumo horario" sheetId="3" r:id="R4edba76ee9454c3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generación PVSyst" sheetId="4" r:id="R7a769f0060494f60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfil PVSyst" sheetId="5" r:id="R13882c0a788f40aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="Ra116970976d24458"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuración" sheetId="2" r:id="R7e8ad242f99e42ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consumo horario" sheetId="3" r:id="R0ef71cc4f9ec40f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generación PVSyst" sheetId="4" r:id="R7eec5dc7fd38493f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Perfil PVSyst" sheetId="5" r:id="Rf67005434b2f4e00"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -65,7 +65,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="14">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -115,6 +115,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF153D35"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF153D35"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF16835C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3CC"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -271,7 +286,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="92">
+  <x:cellXfs count="101">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -434,6 +449,27 @@
     <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="0" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -11940,13 +11976,13 @@
       <x:c r="Z1" s="1"/>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
-      <x:c r="A2" s="80" t="str">
+      <x:c r="A2" s="92" t="str">
         <x:v>Configuración de la planta</x:v>
       </x:c>
-      <x:c r="B2" s="80" t="str">
+      <x:c r="B2" s="92" t="str">
         <x:v>Configuración de la planta</x:v>
       </x:c>
-      <x:c r="C2" s="80" t="str">
+      <x:c r="C2" s="92" t="str">
         <x:v>Configuración de la planta</x:v>
       </x:c>
       <x:c r="D2" s="4" t="str">
@@ -12004,13 +12040,13 @@
       <x:c r="Z3" s="1"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="85" t="str">
+      <x:c r="A4" s="97" t="str">
         <x:v>Campo</x:v>
       </x:c>
-      <x:c r="B4" s="85" t="str">
+      <x:c r="B4" s="97" t="str">
         <x:v>Valor</x:v>
       </x:c>
-      <x:c r="C4" s="85" t="str">
+      <x:c r="C4" s="97" t="str">
         <x:v>Uso en la aplicación</x:v>
       </x:c>
       <x:c r="D4" s="1"/>
@@ -12041,7 +12077,7 @@
       <x:c r="A5" s="63" t="str">
         <x:v>Nombre de la planta</x:v>
       </x:c>
-      <x:c r="B5" s="86" t="str"/>
+      <x:c r="B5" s="98" t="str"/>
       <x:c r="C5" s="63" t="str">
         <x:v>Identifica esta fuente en el selector.</x:v>
       </x:c>
@@ -12073,7 +12109,7 @@
       <x:c r="A6" s="63" t="str">
         <x:v>Año de consumo</x:v>
       </x:c>
-      <x:c r="B6" s="86" t="str"/>
+      <x:c r="B6" s="98" t="str"/>
       <x:c r="C6" s="63" t="str">
         <x:v>Debe coincidir con las fechas de Consumo horario.</x:v>
       </x:c>
@@ -12105,7 +12141,7 @@
       <x:c r="A7" s="63" t="str">
         <x:v>Capacidad FV instalada (kWp)</x:v>
       </x:c>
-      <x:c r="B7" s="87" t="str"/>
+      <x:c r="B7" s="99" t="str"/>
       <x:c r="C7" s="63" t="str">
         <x:v>Referencia para el desempeño técnico.</x:v>
       </x:c>
@@ -12135,11 +12171,11 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="63" t="str">
-        <x:v>Tarifa de energía evitada (COP/kWh)</x:v>
+        <x:v>Tarifa de compra de red (COP/kWh)</x:v>
       </x:c>
-      <x:c r="B8" s="88" t="str"/>
+      <x:c r="B8" s="100" t="str"/>
       <x:c r="C8" s="63" t="str">
-        <x:v>Convierte la desviación energética estimada a COP.</x:v>
+        <x:v>Valora el autoconsumo y la compra residual de energía.</x:v>
       </x:c>
       <x:c r="D8" s="1"/>
       <x:c r="E8" s="1"/>
@@ -12166,9 +12202,13 @@
       <x:c r="Z8" s="1"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="1"/>
-      <x:c r="B9" s="1"/>
-      <x:c r="C9" s="1"/>
+      <x:c r="A9" s="63" t="str">
+        <x:v>Tarifa de exportación (COP/kWh)</x:v>
+      </x:c>
+      <x:c r="B9" s="100" t="str"/>
+      <x:c r="C9" s="63" t="str">
+        <x:v>Opcional. Valora el excedente potencial hacia la red.</x:v>
+      </x:c>
       <x:c r="D9" s="1"/>
       <x:c r="E9" s="1"/>
       <x:c r="F9" s="1"/>
@@ -34515,19 +34555,19 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="80" t="str">
-        <x:v>Producción mensual estimada PVSyst</x:v>
+      <x:c r="A1" s="92" t="str">
+        <x:v>Producción mensual potencial PVSyst</x:v>
       </x:c>
-      <x:c r="B1" s="80" t="str">
-        <x:v>Producción mensual estimada PVSyst</x:v>
+      <x:c r="B1" s="92" t="str">
+        <x:v>Producción mensual potencial PVSyst</x:v>
       </x:c>
-      <x:c r="C1" s="80" t="str">
-        <x:v>Producción mensual estimada PVSyst</x:v>
+      <x:c r="C1" s="92" t="str">
+        <x:v>Producción mensual potencial PVSyst</x:v>
       </x:c>
-      <x:c r="D1" s="80" t="str">
-        <x:v>Producción mensual estimada PVSyst</x:v>
+      <x:c r="D1" s="92" t="str">
+        <x:v>Producción mensual potencial PVSyst</x:v>
       </x:c>
-      <x:c r="E1" s="80"/>
+      <x:c r="E1"/>
       <x:c r="F1" s="1"/>
       <x:c r="G1" s="1"/>
       <x:c r="H1" s="1"/>
@@ -34557,7 +34597,7 @@
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
       <x:c r="D2" s="1"/>
-      <x:c r="E2" s="1"/>
+      <x:c r="E2"/>
       <x:c r="F2" s="1"/>
       <x:c r="G2" s="1"/>
       <x:c r="H2" s="1"/>
@@ -34585,7 +34625,7 @@
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
       <x:c r="D3" s="1"/>
-      <x:c r="E3" s="1"/>
+      <x:c r="E3"/>
       <x:c r="F3" s="1"/>
       <x:c r="G3" s="1"/>
       <x:c r="H3" s="1"/>
@@ -34621,9 +34661,7 @@
       <x:c r="D4" s="12" t="str">
         <x:v>PR (%)</x:v>
       </x:c>
-      <x:c r="E4" s="85" t="str">
-        <x:v>Generación real (kWh)</x:v>
-      </x:c>
+      <x:c r="E4"/>
       <x:c r="F4" s="1"/>
       <x:c r="G4" s="1"/>
       <x:c r="H4" s="1"/>
@@ -34653,7 +34691,7 @@
       <x:c r="B5" s="54"/>
       <x:c r="C5" s="54"/>
       <x:c r="D5" s="55"/>
-      <x:c r="E5" s="91"/>
+      <x:c r="E5"/>
       <x:c r="F5" s="1"/>
       <x:c r="G5" s="1"/>
       <x:c r="H5" s="1"/>
@@ -34683,7 +34721,7 @@
       <x:c r="B6" s="54"/>
       <x:c r="C6" s="54"/>
       <x:c r="D6" s="55"/>
-      <x:c r="E6" s="91"/>
+      <x:c r="E6"/>
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
       <x:c r="H6" s="1"/>
@@ -34713,7 +34751,7 @@
       <x:c r="B7" s="54"/>
       <x:c r="C7" s="54"/>
       <x:c r="D7" s="55"/>
-      <x:c r="E7" s="91"/>
+      <x:c r="E7"/>
       <x:c r="F7" s="1"/>
       <x:c r="G7" s="1"/>
       <x:c r="H7" s="1"/>
@@ -34743,7 +34781,7 @@
       <x:c r="B8" s="54"/>
       <x:c r="C8" s="54"/>
       <x:c r="D8" s="55"/>
-      <x:c r="E8" s="91"/>
+      <x:c r="E8"/>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
       <x:c r="H8" s="1"/>
@@ -34773,7 +34811,7 @@
       <x:c r="B9" s="54"/>
       <x:c r="C9" s="54"/>
       <x:c r="D9" s="55"/>
-      <x:c r="E9" s="91"/>
+      <x:c r="E9"/>
       <x:c r="F9" s="1"/>
       <x:c r="G9" s="1"/>
       <x:c r="H9" s="1"/>
@@ -34803,7 +34841,7 @@
       <x:c r="B10" s="54"/>
       <x:c r="C10" s="54"/>
       <x:c r="D10" s="55"/>
-      <x:c r="E10" s="91"/>
+      <x:c r="E10"/>
       <x:c r="F10" s="1"/>
       <x:c r="G10" s="1"/>
       <x:c r="H10" s="1"/>
@@ -34833,7 +34871,7 @@
       <x:c r="B11" s="54"/>
       <x:c r="C11" s="54"/>
       <x:c r="D11" s="55"/>
-      <x:c r="E11" s="91"/>
+      <x:c r="E11"/>
       <x:c r="F11" s="1"/>
       <x:c r="G11" s="1"/>
       <x:c r="H11" s="1"/>
@@ -34863,7 +34901,7 @@
       <x:c r="B12" s="54"/>
       <x:c r="C12" s="54"/>
       <x:c r="D12" s="55"/>
-      <x:c r="E12" s="91"/>
+      <x:c r="E12"/>
       <x:c r="F12" s="1"/>
       <x:c r="G12" s="1"/>
       <x:c r="H12" s="1"/>
@@ -34893,7 +34931,7 @@
       <x:c r="B13" s="54"/>
       <x:c r="C13" s="54"/>
       <x:c r="D13" s="55"/>
-      <x:c r="E13" s="91"/>
+      <x:c r="E13"/>
       <x:c r="F13" s="1"/>
       <x:c r="G13" s="1"/>
       <x:c r="H13" s="1"/>
@@ -34923,7 +34961,7 @@
       <x:c r="B14" s="54"/>
       <x:c r="C14" s="54"/>
       <x:c r="D14" s="55"/>
-      <x:c r="E14" s="91"/>
+      <x:c r="E14"/>
       <x:c r="F14" s="1"/>
       <x:c r="G14" s="1"/>
       <x:c r="H14" s="1"/>
@@ -34953,7 +34991,7 @@
       <x:c r="B15" s="54"/>
       <x:c r="C15" s="54"/>
       <x:c r="D15" s="55"/>
-      <x:c r="E15" s="91"/>
+      <x:c r="E15"/>
       <x:c r="F15" s="1"/>
       <x:c r="G15" s="1"/>
       <x:c r="H15" s="1"/>
@@ -34983,7 +35021,7 @@
       <x:c r="B16" s="54"/>
       <x:c r="C16" s="54"/>
       <x:c r="D16" s="55"/>
-      <x:c r="E16" s="91"/>
+      <x:c r="E16"/>
       <x:c r="F16" s="1"/>
       <x:c r="G16" s="1"/>
       <x:c r="H16" s="1"/>
@@ -45761,7 +45799,7 @@
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:D2"/>
-    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A1:D1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>